<commit_message>
UAT walkthrough users workbook: responsibilities of every listed persona, flow titles of the Data Migration storyboard, password reset note on the cover
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/UAT/BIBS_UAT_BRD-00_Walkthrough_Users_and_Sign-in_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/UAT/BIBS_UAT_BRD-00_Walkthrough_Users_and_Sign-in_v1.0.xlsx
@@ -3401,7 +3401,11 @@
       </c>
       <c r="D13" s="12" t="n"/>
       <c r="E13" s="12" t="n"/>
-      <c r="F13" s="12" t="n"/>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>Answers requests, submits proposals, decides franchise, bills member changes, uploads policy forms and SOAs, for its own insurer only</t>
+        </is>
+      </c>
       <c r="G13" s="12" t="n"/>
       <c r="H13" s="12" t="inlineStr">
         <is>
@@ -3431,7 +3435,11 @@
       </c>
       <c r="D14" s="12" t="n"/>
       <c r="E14" s="12" t="n"/>
-      <c r="F14" s="12" t="n"/>
+      <c r="F14" s="12" t="inlineStr">
+        <is>
+          <t>Views its programmes and roster, uploads master lists, utilization, member changes and feedback, comments on and confirms the comparative, for its own company only</t>
+        </is>
+      </c>
       <c r="G14" s="12" t="n"/>
       <c r="H14" s="12" t="inlineStr">
         <is>
@@ -7610,7 +7618,11 @@
           <t>BDO Insurance and Reinsurance Brokers, Inc. / Head Office - Makati / Top Management</t>
         </is>
       </c>
-      <c r="F19" s="12" t="n"/>
+      <c r="F19" s="12" t="inlineStr">
+        <is>
+          <t>Approves the Unapplied to Income batches after the Cashiering team lead</t>
+        </is>
+      </c>
       <c r="G19" s="12" t="inlineStr">
         <is>
           <t>Finance › Cashiering › Unapplied to Income</t>
@@ -7780,7 +7792,11 @@
           <t>BDO Insurance and Reinsurance Brokers, Inc. / Head Office - Makati / Marketing - Collection</t>
         </is>
       </c>
-      <c r="F22" s="12" t="n"/>
+      <c r="F22" s="12" t="inlineStr">
+        <is>
+          <t>Legacy PR 2307 Reversal batches (BRD V0.03); finds the migrated items on the PR Worklist</t>
+        </is>
+      </c>
       <c r="G22" s="12" t="inlineStr">
         <is>
           <t>Finance › Collections › PR Worklist</t>
@@ -7838,7 +7854,11 @@
           <t>BDO Insurance and Reinsurance Brokers, Inc. / Head Office - Makati / Marketing - Collection</t>
         </is>
       </c>
-      <c r="F23" s="12" t="n"/>
+      <c r="F23" s="12" t="inlineStr">
+        <is>
+          <t>Reviews and posts the Legacy PR 2307 Reversal batches (BRD V0.03)</t>
+        </is>
+      </c>
       <c r="G23" s="12" t="inlineStr">
         <is>
           <t>Finance › Collections › PR Worklist</t>
@@ -36334,7 +36354,11 @@
           <t>BDO Insurance and Reinsurance Brokers, Inc. / Head Office - Makati / Operations - Cashiering</t>
         </is>
       </c>
-      <c r="F10" s="12" t="n"/>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>Read access and exports; executes the application requests on its Incoming Requests screen</t>
+        </is>
+      </c>
       <c r="G10" s="12" t="inlineStr">
         <is>
           <t>Finance › Cashiering › Incoming Requests</t>
@@ -36678,7 +36702,11 @@
           <t>BDO Insurance and Reinsurance Brokers, Inc. / Head Office - Makati / Operations - Commission Receivables</t>
         </is>
       </c>
-      <c r="F16" s="12" t="n"/>
+      <c r="F16" s="12" t="inlineStr">
+        <is>
+          <t>Confirms the direct payment accounts fully paid to the insurer and bills the commission receivable in Commission Receivables (BRD-2); views the Collections accounts</t>
+        </is>
+      </c>
       <c r="G16" s="12" t="inlineStr">
         <is>
           <t>Finance › Commission Receivables › DP Accounts</t>
@@ -36732,7 +36760,11 @@
           <t>BDO Insurance and Reinsurance Brokers, Inc. / Head Office - Makati / Operations - Commission Receivables</t>
         </is>
       </c>
-      <c r="F17" s="12" t="n"/>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>As the handler, for the team; views the Collections accounts</t>
+        </is>
+      </c>
       <c r="G17" s="12" t="inlineStr">
         <is>
           <t>Finance › Commission Receivables › DP Accounts</t>
@@ -38559,7 +38591,11 @@
           <t>BDO Insurance and Reinsurance Brokers, Inc. / Head Office - Makati / Comptrollership</t>
         </is>
       </c>
-      <c r="F23" s="12" t="n"/>
+      <c r="F23" s="12" t="inlineStr">
+        <is>
+          <t>Read access to journals, reports and closing</t>
+        </is>
+      </c>
       <c r="G23" s="12" t="inlineStr">
         <is>
           <t>Finance › General Ledger › Journals</t>
@@ -38787,7 +38823,11 @@
           <t>BDO Insurance and Reinsurance Brokers, Inc. / Head Office - Makati / Internal Audit</t>
         </is>
       </c>
-      <c r="F27" s="12" t="n"/>
+      <c r="F27" s="12" t="inlineStr">
+        <is>
+          <t>Read access to journals, reports and closing</t>
+        </is>
+      </c>
       <c r="G27" s="12" t="inlineStr">
         <is>
           <t>Reports › Reports › Report Centre</t>

</xml_diff>